<commit_message>
fix(app): wav2vec2 install, quote UI polish, remove easter egg, v1.8.11
Fix native pack ID validation for wav2vec2 KO/EN download, redesign main quote panel, remove logo easter egg.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/nrm-music-quotes.xlsx
+++ b/data/nrm-music-quotes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AIProj\CsTool\NullReferMusic\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2248985-C0C3-4601-814F-9C8E2928C32A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{88EB7D73-9218-4244-B794-1A5A080977EF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="23760" windowHeight="12870" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1350" uniqueCount="885">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1355" uniqueCount="890">
   <si>
     <t>nameKo</t>
   </si>
@@ -2690,6 +2690,26 @@
   </si>
   <si>
     <t>잠은 돈이 없는 거지들이나 자는 것이다.</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>윤현상</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Steven Yoon</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1996 ~</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FUCK YOU</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>안녕하세요.</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -3074,8 +3094,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E270"/>
-  <sheetFormatPr defaultRowHeight="16.5" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E271"/>
+  <sheetFormatPr defaultRowHeight="17.25" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.21875" customWidth="1"/>
     <col min="2" max="2" width="12.21875" customWidth="1"/>
@@ -3084,7 +3104,7 @@
     <col min="5" max="5" width="122.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -3101,7 +3121,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>5</v>
       </c>
@@ -3118,7 +3138,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>5</v>
       </c>
@@ -3135,7 +3155,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>5</v>
       </c>
@@ -3152,7 +3172,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>5</v>
       </c>
@@ -3169,7 +3189,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -3186,7 +3206,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="7" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -3203,7 +3223,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -3220,7 +3240,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>18</v>
       </c>
@@ -3237,7 +3257,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>18</v>
       </c>
@@ -3254,7 +3274,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>29</v>
       </c>
@@ -3271,7 +3291,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>29</v>
       </c>
@@ -3288,7 +3308,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>29</v>
       </c>
@@ -3305,7 +3325,7 @@
         <v>869</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>37</v>
       </c>
@@ -3322,7 +3342,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="15" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>37</v>
       </c>
@@ -3339,7 +3359,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="16" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>37</v>
       </c>
@@ -3356,7 +3376,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>46</v>
       </c>
@@ -3373,7 +3393,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="18" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>46</v>
       </c>
@@ -3390,7 +3410,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="19" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>46</v>
       </c>
@@ -3407,7 +3427,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="20" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>55</v>
       </c>
@@ -3424,7 +3444,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>55</v>
       </c>
@@ -3441,7 +3461,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="22" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>55</v>
       </c>
@@ -3458,7 +3478,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="23" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>55</v>
       </c>
@@ -3475,7 +3495,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="24" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>66</v>
       </c>
@@ -3492,7 +3512,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="25" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>66</v>
       </c>
@@ -3509,7 +3529,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>66</v>
       </c>
@@ -3526,7 +3546,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>75</v>
       </c>
@@ -3543,7 +3563,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="28" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>75</v>
       </c>
@@ -3560,7 +3580,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="29" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>82</v>
       </c>
@@ -3577,7 +3597,7 @@
         <v>870</v>
       </c>
     </row>
-    <row r="30" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>82</v>
       </c>
@@ -3594,7 +3614,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>88</v>
       </c>
@@ -3611,7 +3631,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="32" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -3628,7 +3648,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="33" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>88</v>
       </c>
@@ -3645,7 +3665,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="34" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>97</v>
       </c>
@@ -3662,7 +3682,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="35" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>97</v>
       </c>
@@ -3679,7 +3699,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="36" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>97</v>
       </c>
@@ -3696,7 +3716,7 @@
         <v>105</v>
       </c>
     </row>
-    <row r="37" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>106</v>
       </c>
@@ -3713,7 +3733,7 @@
         <v>110</v>
       </c>
     </row>
-    <row r="38" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>106</v>
       </c>
@@ -3730,7 +3750,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="39" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>113</v>
       </c>
@@ -3747,7 +3767,7 @@
         <v>117</v>
       </c>
     </row>
-    <row r="40" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>113</v>
       </c>
@@ -3764,7 +3784,7 @@
         <v>871</v>
       </c>
     </row>
-    <row r="41" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>113</v>
       </c>
@@ -3781,7 +3801,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="42" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>121</v>
       </c>
@@ -3798,7 +3818,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>121</v>
       </c>
@@ -3815,7 +3835,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="44" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>128</v>
       </c>
@@ -3832,7 +3852,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="45" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>128</v>
       </c>
@@ -3849,7 +3869,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="46" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>135</v>
       </c>
@@ -3866,7 +3886,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="47" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>135</v>
       </c>
@@ -3883,7 +3903,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="48" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>142</v>
       </c>
@@ -3900,7 +3920,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="49" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>147</v>
       </c>
@@ -3917,7 +3937,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="50" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>147</v>
       </c>
@@ -3934,7 +3954,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="51" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>154</v>
       </c>
@@ -3951,7 +3971,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="52" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>159</v>
       </c>
@@ -3968,7 +3988,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="53" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>164</v>
       </c>
@@ -3985,7 +4005,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="54" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>164</v>
       </c>
@@ -4002,7 +4022,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="55" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>164</v>
       </c>
@@ -4019,7 +4039,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="56" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>173</v>
       </c>
@@ -4036,7 +4056,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="57" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>173</v>
       </c>
@@ -4053,7 +4073,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="58" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>173</v>
       </c>
@@ -4070,7 +4090,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="59" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>182</v>
       </c>
@@ -4087,7 +4107,7 @@
         <v>186</v>
       </c>
     </row>
-    <row r="60" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>182</v>
       </c>
@@ -4104,7 +4124,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="61" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>182</v>
       </c>
@@ -4121,7 +4141,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="62" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>191</v>
       </c>
@@ -4138,7 +4158,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="63" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>191</v>
       </c>
@@ -4155,7 +4175,7 @@
         <v>197</v>
       </c>
     </row>
-    <row r="64" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>198</v>
       </c>
@@ -4172,7 +4192,7 @@
         <v>202</v>
       </c>
     </row>
-    <row r="65" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>198</v>
       </c>
@@ -4189,7 +4209,7 @@
         <v>204</v>
       </c>
     </row>
-    <row r="66" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>205</v>
       </c>
@@ -4206,7 +4226,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="67" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>205</v>
       </c>
@@ -4223,7 +4243,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="68" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>205</v>
       </c>
@@ -4240,7 +4260,7 @@
         <v>872</v>
       </c>
     </row>
-    <row r="69" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>213</v>
       </c>
@@ -4257,7 +4277,7 @@
         <v>217</v>
       </c>
     </row>
-    <row r="70" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>218</v>
       </c>
@@ -4274,7 +4294,7 @@
         <v>222</v>
       </c>
     </row>
-    <row r="71" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>218</v>
       </c>
@@ -4291,7 +4311,7 @@
         <v>224</v>
       </c>
     </row>
-    <row r="72" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>218</v>
       </c>
@@ -4308,7 +4328,7 @@
         <v>226</v>
       </c>
     </row>
-    <row r="73" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>218</v>
       </c>
@@ -4325,7 +4345,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="74" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>229</v>
       </c>
@@ -4342,7 +4362,7 @@
         <v>233</v>
       </c>
     </row>
-    <row r="75" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>229</v>
       </c>
@@ -4359,7 +4379,7 @@
         <v>235</v>
       </c>
     </row>
-    <row r="76" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>236</v>
       </c>
@@ -4376,7 +4396,7 @@
         <v>240</v>
       </c>
     </row>
-    <row r="77" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>236</v>
       </c>
@@ -4393,7 +4413,7 @@
         <v>242</v>
       </c>
     </row>
-    <row r="78" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>243</v>
       </c>
@@ -4410,7 +4430,7 @@
         <v>247</v>
       </c>
     </row>
-    <row r="79" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>243</v>
       </c>
@@ -4427,7 +4447,7 @@
         <v>249</v>
       </c>
     </row>
-    <row r="80" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>243</v>
       </c>
@@ -4444,7 +4464,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="81" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>243</v>
       </c>
@@ -4461,7 +4481,7 @@
         <v>253</v>
       </c>
     </row>
-    <row r="82" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>254</v>
       </c>
@@ -4478,7 +4498,7 @@
         <v>258</v>
       </c>
     </row>
-    <row r="83" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>254</v>
       </c>
@@ -4495,7 +4515,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="84" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>254</v>
       </c>
@@ -4512,7 +4532,7 @@
         <v>262</v>
       </c>
     </row>
-    <row r="85" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>263</v>
       </c>
@@ -4529,7 +4549,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="86" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>263</v>
       </c>
@@ -4546,7 +4566,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="87" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>263</v>
       </c>
@@ -4563,7 +4583,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="88" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>272</v>
       </c>
@@ -4580,7 +4600,7 @@
         <v>276</v>
       </c>
     </row>
-    <row r="89" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>272</v>
       </c>
@@ -4597,7 +4617,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="90" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>272</v>
       </c>
@@ -4614,7 +4634,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="91" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>280</v>
       </c>
@@ -4631,7 +4651,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="92" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>280</v>
       </c>
@@ -4648,7 +4668,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="93" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>280</v>
       </c>
@@ -4665,7 +4685,7 @@
         <v>874</v>
       </c>
     </row>
-    <row r="94" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>288</v>
       </c>
@@ -4682,7 +4702,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="95" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>288</v>
       </c>
@@ -4699,7 +4719,7 @@
         <v>294</v>
       </c>
     </row>
-    <row r="96" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>295</v>
       </c>
@@ -4716,7 +4736,7 @@
         <v>298</v>
       </c>
     </row>
-    <row r="97" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>295</v>
       </c>
@@ -4733,7 +4753,7 @@
         <v>875</v>
       </c>
     </row>
-    <row r="98" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>300</v>
       </c>
@@ -4750,7 +4770,7 @@
         <v>304</v>
       </c>
     </row>
-    <row r="99" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>300</v>
       </c>
@@ -4767,7 +4787,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="100" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>307</v>
       </c>
@@ -4784,7 +4804,7 @@
         <v>311</v>
       </c>
     </row>
-    <row r="101" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>307</v>
       </c>
@@ -4801,7 +4821,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="102" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>314</v>
       </c>
@@ -4818,7 +4838,7 @@
         <v>318</v>
       </c>
     </row>
-    <row r="103" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>314</v>
       </c>
@@ -4835,7 +4855,7 @@
         <v>320</v>
       </c>
     </row>
-    <row r="104" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>321</v>
       </c>
@@ -4852,7 +4872,7 @@
         <v>325</v>
       </c>
     </row>
-    <row r="105" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>321</v>
       </c>
@@ -4869,7 +4889,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="106" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>321</v>
       </c>
@@ -4886,7 +4906,7 @@
         <v>329</v>
       </c>
     </row>
-    <row r="107" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>330</v>
       </c>
@@ -4903,7 +4923,7 @@
         <v>334</v>
       </c>
     </row>
-    <row r="108" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>330</v>
       </c>
@@ -4920,7 +4940,7 @@
         <v>336</v>
       </c>
     </row>
-    <row r="109" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>330</v>
       </c>
@@ -4937,7 +4957,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="110" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>339</v>
       </c>
@@ -4954,7 +4974,7 @@
         <v>876</v>
       </c>
     </row>
-    <row r="111" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>339</v>
       </c>
@@ -4971,7 +4991,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="112" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>345</v>
       </c>
@@ -4988,7 +5008,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="113" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>345</v>
       </c>
@@ -5005,7 +5025,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="114" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>352</v>
       </c>
@@ -5022,7 +5042,7 @@
         <v>356</v>
       </c>
     </row>
-    <row r="115" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>352</v>
       </c>
@@ -5039,7 +5059,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="116" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>359</v>
       </c>
@@ -5056,7 +5076,7 @@
         <v>363</v>
       </c>
     </row>
-    <row r="117" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>359</v>
       </c>
@@ -5073,7 +5093,7 @@
         <v>365</v>
       </c>
     </row>
-    <row r="118" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>359</v>
       </c>
@@ -5090,7 +5110,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="119" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>368</v>
       </c>
@@ -5107,7 +5127,7 @@
         <v>372</v>
       </c>
     </row>
-    <row r="120" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>368</v>
       </c>
@@ -5124,7 +5144,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="121" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>368</v>
       </c>
@@ -5141,7 +5161,7 @@
         <v>376</v>
       </c>
     </row>
-    <row r="122" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>368</v>
       </c>
@@ -5158,7 +5178,7 @@
         <v>378</v>
       </c>
     </row>
-    <row r="123" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>379</v>
       </c>
@@ -5175,7 +5195,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="124" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>379</v>
       </c>
@@ -5192,7 +5212,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="125" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>386</v>
       </c>
@@ -5209,7 +5229,7 @@
         <v>390</v>
       </c>
     </row>
-    <row r="126" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>386</v>
       </c>
@@ -5226,7 +5246,7 @@
         <v>392</v>
       </c>
     </row>
-    <row r="127" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>393</v>
       </c>
@@ -5243,7 +5263,7 @@
         <v>397</v>
       </c>
     </row>
-    <row r="128" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>393</v>
       </c>
@@ -5260,7 +5280,7 @@
         <v>399</v>
       </c>
     </row>
-    <row r="129" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>400</v>
       </c>
@@ -5277,7 +5297,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="130" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>400</v>
       </c>
@@ -5294,7 +5314,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="131" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>407</v>
       </c>
@@ -5311,7 +5331,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="132" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>407</v>
       </c>
@@ -5328,7 +5348,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="133" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>414</v>
       </c>
@@ -5345,7 +5365,7 @@
         <v>418</v>
       </c>
     </row>
-    <row r="134" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>419</v>
       </c>
@@ -5362,7 +5382,7 @@
         <v>423</v>
       </c>
     </row>
-    <row r="135" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>424</v>
       </c>
@@ -5379,7 +5399,7 @@
         <v>428</v>
       </c>
     </row>
-    <row r="136" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>429</v>
       </c>
@@ -5396,7 +5416,7 @@
         <v>433</v>
       </c>
     </row>
-    <row r="137" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>434</v>
       </c>
@@ -5413,7 +5433,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="138" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>439</v>
       </c>
@@ -5430,7 +5450,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="139" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>444</v>
       </c>
@@ -5447,7 +5467,7 @@
         <v>448</v>
       </c>
     </row>
-    <row r="140" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>449</v>
       </c>
@@ -5464,7 +5484,7 @@
         <v>453</v>
       </c>
     </row>
-    <row r="141" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>449</v>
       </c>
@@ -5481,7 +5501,7 @@
         <v>455</v>
       </c>
     </row>
-    <row r="142" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>456</v>
       </c>
@@ -5498,7 +5518,7 @@
         <v>460</v>
       </c>
     </row>
-    <row r="143" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>456</v>
       </c>
@@ -5515,7 +5535,7 @@
         <v>462</v>
       </c>
     </row>
-    <row r="144" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>463</v>
       </c>
@@ -5532,7 +5552,7 @@
         <v>467</v>
       </c>
     </row>
-    <row r="145" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>463</v>
       </c>
@@ -5549,7 +5569,7 @@
         <v>469</v>
       </c>
     </row>
-    <row r="146" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>463</v>
       </c>
@@ -5566,7 +5586,7 @@
         <v>471</v>
       </c>
     </row>
-    <row r="147" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>472</v>
       </c>
@@ -5583,7 +5603,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="148" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>472</v>
       </c>
@@ -5600,7 +5620,7 @@
         <v>478</v>
       </c>
     </row>
-    <row r="149" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>472</v>
       </c>
@@ -5617,7 +5637,7 @@
         <v>480</v>
       </c>
     </row>
-    <row r="150" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>481</v>
       </c>
@@ -5634,7 +5654,7 @@
         <v>485</v>
       </c>
     </row>
-    <row r="151" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>481</v>
       </c>
@@ -5651,7 +5671,7 @@
         <v>487</v>
       </c>
     </row>
-    <row r="152" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>488</v>
       </c>
@@ -5668,7 +5688,7 @@
         <v>492</v>
       </c>
     </row>
-    <row r="153" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>488</v>
       </c>
@@ -5685,7 +5705,7 @@
         <v>494</v>
       </c>
     </row>
-    <row r="154" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>495</v>
       </c>
@@ -5702,7 +5722,7 @@
         <v>877</v>
       </c>
     </row>
-    <row r="155" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>495</v>
       </c>
@@ -5719,7 +5739,7 @@
         <v>878</v>
       </c>
     </row>
-    <row r="156" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>500</v>
       </c>
@@ -5736,7 +5756,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="157" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>500</v>
       </c>
@@ -5753,7 +5773,7 @@
         <v>880</v>
       </c>
     </row>
-    <row r="158" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>500</v>
       </c>
@@ -5770,7 +5790,7 @@
         <v>881</v>
       </c>
     </row>
-    <row r="159" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>506</v>
       </c>
@@ -5787,7 +5807,7 @@
         <v>510</v>
       </c>
     </row>
-    <row r="160" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>506</v>
       </c>
@@ -5804,7 +5824,7 @@
         <v>512</v>
       </c>
     </row>
-    <row r="161" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>513</v>
       </c>
@@ -5821,7 +5841,7 @@
         <v>517</v>
       </c>
     </row>
-    <row r="162" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>513</v>
       </c>
@@ -5838,7 +5858,7 @@
         <v>882</v>
       </c>
     </row>
-    <row r="163" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>519</v>
       </c>
@@ -5855,7 +5875,7 @@
         <v>523</v>
       </c>
     </row>
-    <row r="164" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>524</v>
       </c>
@@ -5872,7 +5892,7 @@
         <v>528</v>
       </c>
     </row>
-    <row r="165" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>524</v>
       </c>
@@ -5889,7 +5909,7 @@
         <v>530</v>
       </c>
     </row>
-    <row r="166" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>531</v>
       </c>
@@ -5906,7 +5926,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="167" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="167" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>531</v>
       </c>
@@ -5923,7 +5943,7 @@
         <v>537</v>
       </c>
     </row>
-    <row r="168" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="168" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>538</v>
       </c>
@@ -5940,7 +5960,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="169" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="169" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>543</v>
       </c>
@@ -5957,7 +5977,7 @@
         <v>547</v>
       </c>
     </row>
-    <row r="170" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="170" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>548</v>
       </c>
@@ -5974,7 +5994,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="171" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="171" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>553</v>
       </c>
@@ -5991,7 +6011,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="172" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="172" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>558</v>
       </c>
@@ -6008,7 +6028,7 @@
         <v>883</v>
       </c>
     </row>
-    <row r="173" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="173" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>558</v>
       </c>
@@ -6025,7 +6045,7 @@
         <v>563</v>
       </c>
     </row>
-    <row r="174" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="174" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>558</v>
       </c>
@@ -6042,7 +6062,7 @@
         <v>565</v>
       </c>
     </row>
-    <row r="175" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="175" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>558</v>
       </c>
@@ -6059,7 +6079,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="176" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="176" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>568</v>
       </c>
@@ -6076,7 +6096,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="177" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="177" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>568</v>
       </c>
@@ -6093,7 +6113,7 @@
         <v>574</v>
       </c>
     </row>
-    <row r="178" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="178" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>568</v>
       </c>
@@ -6110,7 +6130,7 @@
         <v>576</v>
       </c>
     </row>
-    <row r="179" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="179" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>568</v>
       </c>
@@ -6127,7 +6147,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="180" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="180" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>579</v>
       </c>
@@ -6144,7 +6164,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="181" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="181" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>579</v>
       </c>
@@ -6161,7 +6181,7 @@
         <v>585</v>
       </c>
     </row>
-    <row r="182" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="182" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>579</v>
       </c>
@@ -6178,7 +6198,7 @@
         <v>587</v>
       </c>
     </row>
-    <row r="183" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="183" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>588</v>
       </c>
@@ -6195,7 +6215,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="184" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="184" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>588</v>
       </c>
@@ -6212,7 +6232,7 @@
         <v>593</v>
       </c>
     </row>
-    <row r="185" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="185" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>588</v>
       </c>
@@ -6229,7 +6249,7 @@
         <v>595</v>
       </c>
     </row>
-    <row r="186" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="186" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>588</v>
       </c>
@@ -6246,7 +6266,7 @@
         <v>597</v>
       </c>
     </row>
-    <row r="187" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="187" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>598</v>
       </c>
@@ -6263,7 +6283,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="188" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="188" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>598</v>
       </c>
@@ -6280,7 +6300,7 @@
         <v>604</v>
       </c>
     </row>
-    <row r="189" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="189" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>598</v>
       </c>
@@ -6297,7 +6317,7 @@
         <v>606</v>
       </c>
     </row>
-    <row r="190" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="190" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>598</v>
       </c>
@@ -6314,7 +6334,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="191" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="191" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>609</v>
       </c>
@@ -6331,7 +6351,7 @@
         <v>613</v>
       </c>
     </row>
-    <row r="192" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="192" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>609</v>
       </c>
@@ -6348,7 +6368,7 @@
         <v>615</v>
       </c>
     </row>
-    <row r="193" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="193" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>609</v>
       </c>
@@ -6365,7 +6385,7 @@
         <v>617</v>
       </c>
     </row>
-    <row r="194" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="194" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>618</v>
       </c>
@@ -6382,7 +6402,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="195" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="195" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>618</v>
       </c>
@@ -6399,7 +6419,7 @@
         <v>624</v>
       </c>
     </row>
-    <row r="196" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="196" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>618</v>
       </c>
@@ -6416,7 +6436,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="197" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="197" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>627</v>
       </c>
@@ -6433,7 +6453,7 @@
         <v>630</v>
       </c>
     </row>
-    <row r="198" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="198" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>627</v>
       </c>
@@ -6450,7 +6470,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="199" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="199" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>633</v>
       </c>
@@ -6467,7 +6487,7 @@
         <v>636</v>
       </c>
     </row>
-    <row r="200" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="200" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>633</v>
       </c>
@@ -6484,7 +6504,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="201" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="201" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>639</v>
       </c>
@@ -6501,7 +6521,7 @@
         <v>643</v>
       </c>
     </row>
-    <row r="202" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="202" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>639</v>
       </c>
@@ -6518,7 +6538,7 @@
         <v>884</v>
       </c>
     </row>
-    <row r="203" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="203" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>639</v>
       </c>
@@ -6535,7 +6555,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="204" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="204" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>647</v>
       </c>
@@ -6552,7 +6572,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="205" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="205" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>647</v>
       </c>
@@ -6569,7 +6589,7 @@
         <v>653</v>
       </c>
     </row>
-    <row r="206" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="206" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>647</v>
       </c>
@@ -6586,7 +6606,7 @@
         <v>655</v>
       </c>
     </row>
-    <row r="207" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="207" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>656</v>
       </c>
@@ -6603,7 +6623,7 @@
         <v>660</v>
       </c>
     </row>
-    <row r="208" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="208" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>656</v>
       </c>
@@ -6620,7 +6640,7 @@
         <v>662</v>
       </c>
     </row>
-    <row r="209" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="209" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>656</v>
       </c>
@@ -6637,7 +6657,7 @@
         <v>664</v>
       </c>
     </row>
-    <row r="210" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="210" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>665</v>
       </c>
@@ -6654,7 +6674,7 @@
         <v>669</v>
       </c>
     </row>
-    <row r="211" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="211" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>665</v>
       </c>
@@ -6671,7 +6691,7 @@
         <v>671</v>
       </c>
     </row>
-    <row r="212" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="212" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>665</v>
       </c>
@@ -6688,7 +6708,7 @@
         <v>673</v>
       </c>
     </row>
-    <row r="213" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="213" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>674</v>
       </c>
@@ -6705,7 +6725,7 @@
         <v>678</v>
       </c>
     </row>
-    <row r="214" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="214" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>674</v>
       </c>
@@ -6722,7 +6742,7 @@
         <v>680</v>
       </c>
     </row>
-    <row r="215" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="215" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>674</v>
       </c>
@@ -6739,7 +6759,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="216" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="216" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>683</v>
       </c>
@@ -6756,7 +6776,7 @@
         <v>687</v>
       </c>
     </row>
-    <row r="217" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="217" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>683</v>
       </c>
@@ -6773,7 +6793,7 @@
         <v>689</v>
       </c>
     </row>
-    <row r="218" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="218" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>683</v>
       </c>
@@ -6790,7 +6810,7 @@
         <v>691</v>
       </c>
     </row>
-    <row r="219" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="219" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>692</v>
       </c>
@@ -6807,7 +6827,7 @@
         <v>695</v>
       </c>
     </row>
-    <row r="220" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="220" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>692</v>
       </c>
@@ -6824,7 +6844,7 @@
         <v>697</v>
       </c>
     </row>
-    <row r="221" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="221" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>698</v>
       </c>
@@ -6841,7 +6861,7 @@
         <v>702</v>
       </c>
     </row>
-    <row r="222" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="222" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>698</v>
       </c>
@@ -6858,7 +6878,7 @@
         <v>704</v>
       </c>
     </row>
-    <row r="223" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="223" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>705</v>
       </c>
@@ -6875,7 +6895,7 @@
         <v>709</v>
       </c>
     </row>
-    <row r="224" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="224" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>705</v>
       </c>
@@ -6892,7 +6912,7 @@
         <v>711</v>
       </c>
     </row>
-    <row r="225" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="225" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>712</v>
       </c>
@@ -6909,7 +6929,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="226" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="226" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>712</v>
       </c>
@@ -6926,7 +6946,7 @@
         <v>717</v>
       </c>
     </row>
-    <row r="227" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="227" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>718</v>
       </c>
@@ -6943,7 +6963,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="228" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="228" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>718</v>
       </c>
@@ -6960,7 +6980,7 @@
         <v>723</v>
       </c>
     </row>
-    <row r="229" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="229" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>724</v>
       </c>
@@ -6977,7 +6997,7 @@
         <v>727</v>
       </c>
     </row>
-    <row r="230" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="230" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>724</v>
       </c>
@@ -6994,7 +7014,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="231" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="231" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>724</v>
       </c>
@@ -7011,7 +7031,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="232" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="232" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>732</v>
       </c>
@@ -7028,7 +7048,7 @@
         <v>736</v>
       </c>
     </row>
-    <row r="233" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="233" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>732</v>
       </c>
@@ -7045,7 +7065,7 @@
         <v>738</v>
       </c>
     </row>
-    <row r="234" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="234" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>739</v>
       </c>
@@ -7062,7 +7082,7 @@
         <v>742</v>
       </c>
     </row>
-    <row r="235" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="235" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>739</v>
       </c>
@@ -7079,7 +7099,7 @@
         <v>744</v>
       </c>
     </row>
-    <row r="236" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="236" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A236" t="s">
         <v>745</v>
       </c>
@@ -7096,7 +7116,7 @@
         <v>748</v>
       </c>
     </row>
-    <row r="237" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="237" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A237" t="s">
         <v>745</v>
       </c>
@@ -7113,7 +7133,7 @@
         <v>750</v>
       </c>
     </row>
-    <row r="238" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="238" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A238" t="s">
         <v>751</v>
       </c>
@@ -7130,7 +7150,7 @@
         <v>755</v>
       </c>
     </row>
-    <row r="239" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="239" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A239" t="s">
         <v>756</v>
       </c>
@@ -7147,7 +7167,7 @@
         <v>759</v>
       </c>
     </row>
-    <row r="240" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="240" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A240" t="s">
         <v>756</v>
       </c>
@@ -7164,7 +7184,7 @@
         <v>761</v>
       </c>
     </row>
-    <row r="241" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="241" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A241" t="s">
         <v>762</v>
       </c>
@@ -7181,7 +7201,7 @@
         <v>765</v>
       </c>
     </row>
-    <row r="242" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="242" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A242" t="s">
         <v>762</v>
       </c>
@@ -7198,7 +7218,7 @@
         <v>767</v>
       </c>
     </row>
-    <row r="243" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="243" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A243" t="s">
         <v>762</v>
       </c>
@@ -7215,7 +7235,7 @@
         <v>769</v>
       </c>
     </row>
-    <row r="244" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="244" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A244" t="s">
         <v>770</v>
       </c>
@@ -7232,7 +7252,7 @@
         <v>773</v>
       </c>
     </row>
-    <row r="245" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="245" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A245" t="s">
         <v>774</v>
       </c>
@@ -7249,7 +7269,7 @@
         <v>777</v>
       </c>
     </row>
-    <row r="246" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="246" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A246" t="s">
         <v>774</v>
       </c>
@@ -7266,7 +7286,7 @@
         <v>779</v>
       </c>
     </row>
-    <row r="247" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="247" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A247" t="s">
         <v>780</v>
       </c>
@@ -7283,7 +7303,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="248" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="248" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A248" t="s">
         <v>780</v>
       </c>
@@ -7300,7 +7320,7 @@
         <v>786</v>
       </c>
     </row>
-    <row r="249" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="249" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A249" t="s">
         <v>787</v>
       </c>
@@ -7317,7 +7337,7 @@
         <v>790</v>
       </c>
     </row>
-    <row r="250" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="250" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A250" t="s">
         <v>787</v>
       </c>
@@ -7334,7 +7354,7 @@
         <v>792</v>
       </c>
     </row>
-    <row r="251" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="251" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A251" t="s">
         <v>793</v>
       </c>
@@ -7351,7 +7371,7 @@
         <v>796</v>
       </c>
     </row>
-    <row r="252" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="252" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A252" t="s">
         <v>793</v>
       </c>
@@ -7368,7 +7388,7 @@
         <v>798</v>
       </c>
     </row>
-    <row r="253" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="253" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A253" t="s">
         <v>799</v>
       </c>
@@ -7385,7 +7405,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="254" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="254" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A254" t="s">
         <v>804</v>
       </c>
@@ -7402,7 +7422,7 @@
         <v>807</v>
       </c>
     </row>
-    <row r="255" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="255" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A255" t="s">
         <v>808</v>
       </c>
@@ -7419,7 +7439,7 @@
         <v>812</v>
       </c>
     </row>
-    <row r="256" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="256" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A256" t="s">
         <v>808</v>
       </c>
@@ -7436,7 +7456,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="257" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="257" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A257" t="s">
         <v>815</v>
       </c>
@@ -7453,7 +7473,7 @@
         <v>818</v>
       </c>
     </row>
-    <row r="258" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="258" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A258" t="s">
         <v>819</v>
       </c>
@@ -7470,7 +7490,7 @@
         <v>822</v>
       </c>
     </row>
-    <row r="259" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="259" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A259" t="s">
         <v>819</v>
       </c>
@@ -7487,7 +7507,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="260" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="260" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A260" t="s">
         <v>825</v>
       </c>
@@ -7504,7 +7524,7 @@
         <v>828</v>
       </c>
     </row>
-    <row r="261" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="261" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A261" t="s">
         <v>829</v>
       </c>
@@ -7521,7 +7541,7 @@
         <v>832</v>
       </c>
     </row>
-    <row r="262" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="262" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A262" t="s">
         <v>833</v>
       </c>
@@ -7538,7 +7558,7 @@
         <v>837</v>
       </c>
     </row>
-    <row r="263" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="263" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A263" t="s">
         <v>833</v>
       </c>
@@ -7555,7 +7575,7 @@
         <v>839</v>
       </c>
     </row>
-    <row r="264" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="264" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A264" t="s">
         <v>840</v>
       </c>
@@ -7572,7 +7592,7 @@
         <v>843</v>
       </c>
     </row>
-    <row r="265" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="265" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A265" t="s">
         <v>844</v>
       </c>
@@ -7589,7 +7609,7 @@
         <v>847</v>
       </c>
     </row>
-    <row r="266" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="266" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A266" t="s">
         <v>848</v>
       </c>
@@ -7606,7 +7626,7 @@
         <v>852</v>
       </c>
     </row>
-    <row r="267" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="267" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A267" t="s">
         <v>853</v>
       </c>
@@ -7623,7 +7643,7 @@
         <v>857</v>
       </c>
     </row>
-    <row r="268" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="268" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A268" t="s">
         <v>853</v>
       </c>
@@ -7640,7 +7660,7 @@
         <v>859</v>
       </c>
     </row>
-    <row r="269" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="269" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A269" t="s">
         <v>860</v>
       </c>
@@ -7657,7 +7677,7 @@
         <v>863</v>
       </c>
     </row>
-    <row r="270" spans="1:5" ht="17.25" x14ac:dyDescent="0.3">
+    <row r="270" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A270" t="s">
         <v>864</v>
       </c>
@@ -7672,6 +7692,23 @@
       </c>
       <c r="E270" t="s">
         <v>868</v>
+      </c>
+    </row>
+    <row r="271" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A271" t="s">
+        <v>885</v>
+      </c>
+      <c r="B271" t="s">
+        <v>886</v>
+      </c>
+      <c r="C271" t="s">
+        <v>887</v>
+      </c>
+      <c r="D271" t="s">
+        <v>888</v>
+      </c>
+      <c r="E271" t="s">
+        <v>889</v>
       </c>
     </row>
   </sheetData>

</xml_diff>